<commit_message>
feat: add tenant registry generation script and related files
- Introduced `generate-registry.ts` to process tenant and payment data from Excel files and generate a JSON registry.
- Added `tennants-registery.model.ts` for type definitions related to tenant data.
- Created `package.json` and `package-lock.json` for project dependencies and scripts.
- Added TypeScript configuration in `tsconfig.json` for project compilation settings.
- Included Excel files `tennants-list.xlsx` and `payment-history.xlsx` for input data.
- Updated `tennants-registery.json` to include a new tenant mapping.
</commit_message>
<xml_diff>
--- a/inputs/tennants-list.xlsx
+++ b/inputs/tennants-list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Courses\Consult-2605-Shidav\house-commity-payments-with-ai\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59AB99AE-C98F-4245-8394-742BE70722BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18DADA1A-5970-46CF-A045-1BD39D6C48D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27120" yWindow="900" windowWidth="25200" windowHeight="19470" xr2:uid="{F50B43FA-9176-478C-A438-A9922A4BE028}"/>
+    <workbookView xWindow="29850" yWindow="120" windowWidth="25200" windowHeight="19470" xr2:uid="{F50B43FA-9176-478C-A438-A9922A4BE028}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: update tenant registry and payment history files with new entries and improved data handling
</commit_message>
<xml_diff>
--- a/inputs/tennants-list.xlsx
+++ b/inputs/tennants-list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Courses\Consult-2605-Shidav\house-commity-payments-with-ai\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18DADA1A-5970-46CF-A045-1BD39D6C48D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D8D21A2-85FA-4034-BBD8-67EEFA96B2B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29850" yWindow="120" windowWidth="25200" windowHeight="19470" xr2:uid="{F50B43FA-9176-478C-A438-A9922A4BE028}"/>
+    <workbookView xWindow="1650" yWindow="1290" windowWidth="25200" windowHeight="19470" xr2:uid="{F50B43FA-9176-478C-A438-A9922A4BE028}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
   <si>
     <t>Appt</t>
   </si>
@@ -111,6 +111,15 @@
   </si>
   <si>
     <t>Einat@test.co.il</t>
+  </si>
+  <si>
+    <t>אדם סנדלר</t>
+  </si>
+  <si>
+    <t>054-898546</t>
+  </si>
+  <si>
+    <t>adam@test.co.il</t>
   </si>
 </sst>
 </file>
@@ -326,16 +335,10 @@
       <sheetName val="חישוב שטח"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0">
+      <sheetData sheetId="0" refreshError="1">
         <row r="2">
           <cell r="A2">
             <v>7</v>
-          </cell>
-          <cell r="B2">
-            <v>2</v>
-          </cell>
-          <cell r="E2" t="str">
-            <v xml:space="preserve"> </v>
           </cell>
           <cell r="H2" t="str">
             <v xml:space="preserve"> </v>
@@ -343,28 +346,19 @@
           <cell r="I2" t="str">
             <v xml:space="preserve"> </v>
           </cell>
-          <cell r="J2" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
         </row>
         <row r="3">
-          <cell r="A3">
-            <v>8</v>
-          </cell>
-          <cell r="E3" t="str">
-            <v xml:space="preserve"> </v>
-          </cell>
           <cell r="I3" t="str">
             <v xml:space="preserve"> </v>
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -667,10 +661,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46491BBB-1A84-4E53-AADA-65F913860908}">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19.42578125" customWidth="1"/>
+    <col min="8" max="8" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="9" bestFit="1" customWidth="1"/>
   </cols>
@@ -718,11 +717,9 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="7">
-        <f>[1]North!A2</f>
         <v>7</v>
       </c>
       <c r="B2" s="7">
-        <f>[1]North!B2</f>
         <v>2</v>
       </c>
       <c r="C2" s="8" t="s">
@@ -731,10 +728,7 @@
       <c r="D2" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="7" t="str">
-        <f>[1]North!E2</f>
-        <v xml:space="preserve"> </v>
-      </c>
+      <c r="E2" s="7"/>
       <c r="F2" s="13" t="s">
         <v>17</v>
       </c>
@@ -749,10 +743,7 @@
         <f>[1]North!I2</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="J2" s="9" t="str">
-        <f>[1]North!J2</f>
-        <v xml:space="preserve"> </v>
-      </c>
+      <c r="J2" s="9"/>
       <c r="K2" s="10">
         <v>1467</v>
       </c>
@@ -765,7 +756,6 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="7">
-        <f>[1]North!A3</f>
         <v>8</v>
       </c>
       <c r="B3" s="7">
@@ -777,10 +767,7 @@
       <c r="D3" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="12" t="str">
-        <f>[1]North!E3</f>
-        <v xml:space="preserve"> </v>
-      </c>
+      <c r="E3" s="12"/>
       <c r="F3" s="14" t="s">
         <v>18</v>
       </c>
@@ -804,6 +791,41 @@
         <v>1050</v>
       </c>
       <c r="M3" s="11">
+        <v>130.69999999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="7">
+        <v>10</v>
+      </c>
+      <c r="B4" s="7">
+        <v>3</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" s="12"/>
+      <c r="F4" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="I4" s="12"/>
+      <c r="J4" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" s="10">
+        <v>2640</v>
+      </c>
+      <c r="L4" s="10">
+        <v>1050</v>
+      </c>
+      <c r="M4" s="11">
         <v>130.69999999999999</v>
       </c>
     </row>
@@ -812,6 +834,8 @@
     <hyperlink ref="F2" r:id="rId1" xr:uid="{36A81F31-71C0-46D7-AD42-058615C4E513}"/>
     <hyperlink ref="F3" r:id="rId2" xr:uid="{DE710013-211B-40F4-8407-29B05BDF7663}"/>
     <hyperlink ref="J3" r:id="rId3" xr:uid="{CF1A19A3-768E-4AB0-BC83-48106A3AEA7B}"/>
+    <hyperlink ref="F4" r:id="rId4" xr:uid="{B5FFAD95-D733-47A8-B6B2-7A5D17ECADA8}"/>
+    <hyperlink ref="J4" r:id="rId5" xr:uid="{637CE855-97EF-444B-8701-2B8FE16AF1E9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: enhance tenant registry with apartment details including rent and renovation fund amounts
</commit_message>
<xml_diff>
--- a/inputs/tennants-list.xlsx
+++ b/inputs/tennants-list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Courses\Consult-2605-Shidav\house-commity-payments-with-ai\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D8D21A2-85FA-4034-BBD8-67EEFA96B2B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDE17FCC-0206-41D9-A596-C3D57F61EB1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1650" yWindow="1290" windowWidth="25200" windowHeight="19470" xr2:uid="{F50B43FA-9176-478C-A438-A9922A4BE028}"/>
+    <workbookView xWindow="7335" yWindow="1410" windowWidth="21630" windowHeight="19470" xr2:uid="{F50B43FA-9176-478C-A438-A9922A4BE028}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -661,7 +661,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46491BBB-1A84-4E53-AADA-65F913860908}">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
@@ -796,29 +796,21 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="7">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B4" s="7">
         <v>3</v>
       </c>
-      <c r="C4" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>24</v>
-      </c>
+      <c r="C4" s="8"/>
+      <c r="D4" s="12"/>
       <c r="E4" s="12"/>
-      <c r="F4" s="14" t="s">
-        <v>25</v>
-      </c>
+      <c r="F4" s="14"/>
       <c r="G4" s="12"/>
       <c r="H4" s="12" t="s">
         <v>21</v>
       </c>
       <c r="I4" s="12"/>
-      <c r="J4" s="14" t="s">
-        <v>22</v>
-      </c>
+      <c r="J4" s="14"/>
       <c r="K4" s="10">
         <v>2640</v>
       </c>
@@ -826,6 +818,39 @@
         <v>1050</v>
       </c>
       <c r="M4" s="11">
+        <v>130.69999999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" s="7">
+        <v>10</v>
+      </c>
+      <c r="B5" s="7">
+        <v>3</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" s="12"/>
+      <c r="F5" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" s="12"/>
+      <c r="H5" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="I5" s="12"/>
+      <c r="J5" s="14"/>
+      <c r="K5" s="10">
+        <v>2640</v>
+      </c>
+      <c r="L5" s="10">
+        <v>1050</v>
+      </c>
+      <c r="M5" s="11">
         <v>130.69999999999999</v>
       </c>
     </row>
@@ -834,8 +859,7 @@
     <hyperlink ref="F2" r:id="rId1" xr:uid="{36A81F31-71C0-46D7-AD42-058615C4E513}"/>
     <hyperlink ref="F3" r:id="rId2" xr:uid="{DE710013-211B-40F4-8407-29B05BDF7663}"/>
     <hyperlink ref="J3" r:id="rId3" xr:uid="{CF1A19A3-768E-4AB0-BC83-48106A3AEA7B}"/>
-    <hyperlink ref="F4" r:id="rId4" xr:uid="{B5FFAD95-D733-47A8-B6B2-7A5D17ECADA8}"/>
-    <hyperlink ref="J4" r:id="rId5" xr:uid="{637CE855-97EF-444B-8701-2B8FE16AF1E9}"/>
+    <hyperlink ref="F5" r:id="rId4" xr:uid="{B5FFAD95-D733-47A8-B6B2-7A5D17ECADA8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>